<commit_message>
feat: complete deterministic PDF extraction P1
</commit_message>
<xml_diff>
--- a/data/2025/07-botosani/35731-botosani/budget_file.xlsx
+++ b/data/2025/07-botosani/35731-botosani/budget_file.xlsx
@@ -60,11 +60,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +438,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -477,7 +480,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL 2026</t>
+          <t>TOTAL 2025</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -500,7 +503,11 @@
       <c r="E2" t="n">
         <v>2</v>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G2" s="3" t="n">
         <v>42303</v>
       </c>
@@ -510,7 +517,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="30" customHeight="1">
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>- cheltuieli de personal aparatul de specialitate al primarului, consilieri locali și aparatul Consiliului Local</t>
@@ -519,7 +526,11 @@
       <c r="E3" t="n">
         <v>2</v>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G3" s="3" t="n">
         <v>28749</v>
       </c>
@@ -529,16 +540,20 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="75" customHeight="1">
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>- bunuri si servicii - cheltuielile curente de întreținere și funcționare a spațiilor unde îşi desfăşoară activitatea personalul Primăriei Municipiului Botoşani (iluminat și încălzire, materiale de întreținere și curățenie, apă-canal, telefoane, furnituri de birou, service programe informatice, mentenanță, costuri pentru medicina muncii).</t>
+          <t>- bunuri si servici - cheltuielile curente de întreținere și funcționare a spațiilor unde îşi desfăşoară activitatea personalul Primăriei Municipiului Botoşani (iluminat și încălzire, materiale de întreținere și curățenie, apã-canal, telefoane, furnituri de birou, service programe informatice, mentenanță, costuri pentru medicina muncii).</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>2</v>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G4" s="3" t="n">
         <v>4225</v>
       </c>
@@ -557,7 +572,11 @@
       <c r="E5" t="n">
         <v>2</v>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="n">
         <v>285</v>
       </c>
@@ -576,7 +595,11 @@
       <c r="E6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="n">
         <v>9044</v>
       </c>
@@ -595,7 +618,11 @@
       <c r="E7" t="n">
         <v>2</v>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G7" s="3" t="n">
         <v>4215.5</v>
       </c>
@@ -605,7 +632,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="30" customHeight="1">
       <c r="C8" s="2" t="inlineStr">
         <is>
           <t>- cheltuieli de personal Serviciul Public Comunitar de Evidență a Persoanelor</t>
@@ -614,7 +641,11 @@
       <c r="E8" t="n">
         <v>2</v>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G8" s="3" t="n">
         <v>2500.5</v>
       </c>
@@ -624,7 +655,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="30" customHeight="1">
       <c r="C9" s="2" t="inlineStr">
         <is>
           <t>- bunuri si servicii Serviciul Public Comunitar de Evidență a Persoanelor</t>
@@ -633,7 +664,11 @@
       <c r="E9" t="n">
         <v>2</v>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G9" s="3" t="n">
         <v>215</v>
       </c>
@@ -643,16 +678,20 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="75" customHeight="1">
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>- cotizații AsociațiaMunicipiilor, Zona Metropolitană, Asociația G.A.L., sprijin viager pentru persoanele care au împlinit vârsta de 85 de ani, sume acordate pentru cuplurile care au împlinit 50 respectiv 60 de ani de căsătorie, executarea silită a creanțelor bugetare, oraganizare evenimente cu ocazia zilei oraşului, zilei de 1 iunie, sărbători de iarnă</t>
+          <t>- cotizații Asociația Municipiilor, Zona Metropolitană, Asociația G.A.L., sprijin viager pentru persoanele care au împlinit vârsta de 85 de ani, sume acordate pentru cuplurile care au împlinit 50 respectiv 60 de ani de căsătorie, executarea silită a creanțelor bugetare, oraganizare evenimente cu ocazia zilei oraşului, zilei de 1 iunie, sărbători de iarnă</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>2</v>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G10" s="3" t="n">
         <v>1500</v>
       </c>
@@ -671,7 +710,11 @@
       <c r="E11" t="n">
         <v>2</v>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G11" s="3" t="n">
         <v>5</v>
       </c>
@@ -690,7 +733,11 @@
       <c r="E12" t="n">
         <v>2</v>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G12" s="3" t="n">
         <v>9725</v>
       </c>
@@ -709,7 +756,11 @@
       <c r="E13" t="n">
         <v>2</v>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G13" s="3" t="n">
         <v>9725</v>
       </c>
@@ -728,7 +779,11 @@
       <c r="E14" t="n">
         <v>2</v>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G14" s="3" t="n">
         <v>11172.25</v>
       </c>
@@ -738,7 +793,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="30" customHeight="1">
       <c r="C15" s="2" t="inlineStr">
         <is>
           <t>- cheltuieli de personal Serviciul Voluntar pentru Situații de Urgență</t>
@@ -747,7 +802,11 @@
       <c r="E15" t="n">
         <v>2</v>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G15" s="3" t="n">
         <v>140</v>
       </c>
@@ -757,7 +816,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="30" customHeight="1">
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>- bunuri si servicii Serviciul Voluntar pentru Situații de Urgență</t>
@@ -766,7 +825,11 @@
       <c r="E16" t="n">
         <v>2</v>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G16" s="3" t="n">
         <v>43</v>
       </c>
@@ -776,7 +839,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="30" customHeight="1">
       <c r="C17" s="2" t="inlineStr">
         <is>
           <t>- transferuri pentru Poliția Locală (în completarea veniturilor proprii ale instituției)</t>
@@ -785,7 +848,11 @@
       <c r="E17" t="n">
         <v>2</v>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G17" s="3" t="n">
         <v>10989.25</v>
       </c>
@@ -798,13 +865,17 @@
     <row r="18">
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>ÎNVÅTÄMÂNT -total, din care:</t>
+          <t>ÎNVÅTÅMÂNT -total, din care:</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>2</v>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G18" s="3" t="n">
         <v>37388.52</v>
       </c>
@@ -814,7 +885,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="30" customHeight="1">
       <c r="C19" s="2" t="inlineStr">
         <is>
           <t>- finantare de bază în baza costului pe elev și transport elevi</t>
@@ -823,7 +894,11 @@
       <c r="E19" t="n">
         <v>2</v>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G19" s="3" t="n">
         <v>20421</v>
       </c>
@@ -842,7 +917,11 @@
       <c r="E20" t="n">
         <v>2</v>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G20" s="3" t="n">
         <v>2266.52</v>
       </c>
@@ -852,7 +931,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="45" customHeight="1">
       <c r="C21" s="2" t="inlineStr">
         <is>
           <t>- tichete grădiniță - finanțarea drepturilor stabilite de Legea nr.248/2015 privind stimularea participării în învățământul preşcolar a copiilor provenind din familii defavorizate</t>
@@ -861,7 +940,11 @@
       <c r="E21" t="n">
         <v>2</v>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G21" s="3" t="n">
         <v>120</v>
       </c>
@@ -871,7 +954,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="30" customHeight="1">
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>- finantare invatamant particular acreditat în baza costului standard pe elev</t>
@@ -880,7 +963,11 @@
       <c r="E22" t="n">
         <v>2</v>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G22" s="3" t="n">
         <v>7848</v>
       </c>
@@ -890,16 +977,20 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="75" customHeight="1">
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>- finanțarea drepturilor copilor cu cerințe educaționale speciale integrați în învățământul de masă, prevăzute la lit.A din Anexa la HG 904/2014 privind stabilirea limitelor minime de cheltuieli aferente drepturilor prevăzute la art.129 alin(1) din Legea 272/2004 privind protecția și promovarea drepturilor copiilor</t>
+          <t>- finanțarea drepturilor copiilor cu cerințe educaționale speciale integrați în învățământul de masă, prevăzute la lit.A din Anexa la HG 904/2014 privind stabilirea limitelor minime de cheltuieli aferente drepturilor prevăzute la art.129 alin(1) din Legea 272/2004 privind protecția și promovarea drepturilor copiilor</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>3</v>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G23" s="3" t="n">
         <v>2649</v>
       </c>
@@ -918,7 +1009,11 @@
       <c r="E24" t="n">
         <v>3</v>
       </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G24" s="3" t="n">
         <v>3357</v>
       </c>
@@ -928,7 +1023,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="30" customHeight="1">
       <c r="C25" s="2" t="inlineStr">
         <is>
           <t>- asociatii si fundatii (Asociația Il Girotondo cu care Consiliul Local este partener)</t>
@@ -937,7 +1032,11 @@
       <c r="E25" t="n">
         <v>3</v>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G25" s="3" t="n">
         <v>727</v>
       </c>
@@ -956,7 +1055,11 @@
       <c r="E26" t="n">
         <v>3</v>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G26" s="3" t="n">
         <v>9104.4</v>
       </c>
@@ -966,7 +1069,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="60" customHeight="1">
       <c r="C27" s="2" t="inlineStr">
         <is>
           <t>- cheltuieli de personal finanțarea personalului cabinetelor medicale şcolare și cabinete stomatologice care funcționează în instituțiile de învățământ și a asistenței medicale comunitare</t>
@@ -975,7 +1078,11 @@
       <c r="E27" t="n">
         <v>3</v>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G27" s="3" t="n">
         <v>8736.5</v>
       </c>
@@ -985,16 +1092,20 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="30" customHeight="1">
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>- bunuri si servicii cabinete medicale școlare și cabinete stomatologice care funcționează în instituțiile de învățământ</t>
+          <t>- bunuri si servicii cabinete medicale şcolare și cabinete stomatologice care funcționează în instituțiile de învățământ</t>
         </is>
       </c>
       <c r="E28" t="n">
         <v>3</v>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G28" s="3" t="n">
         <v>280.4</v>
       </c>
@@ -1004,7 +1115,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="30" customHeight="1">
       <c r="C29" s="2" t="inlineStr">
         <is>
           <t>- contribuție persoane cu handicap neangajate* cabinete şcolare</t>
@@ -1013,7 +1124,11 @@
       <c r="E29" t="n">
         <v>3</v>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G29" s="3" t="n">
         <v>87.5</v>
       </c>
@@ -1032,7 +1147,11 @@
       <c r="E30" t="n">
         <v>3</v>
       </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G30" s="3" t="n">
         <v>26337.4</v>
       </c>
@@ -1051,7 +1170,11 @@
       <c r="E31" t="n">
         <v>3</v>
       </c>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G31" s="3" t="n">
         <v>432.25</v>
       </c>
@@ -1070,7 +1193,11 @@
       <c r="E32" t="n">
         <v>3</v>
       </c>
-      <c r="F32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G32" s="3" t="n">
         <v>333.35</v>
       </c>
@@ -1080,7 +1207,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="30" customHeight="1">
       <c r="C33" s="2" t="inlineStr">
         <is>
           <t>- Premiul național de poezie "M. Eminescu”, comisii evaluare management instituții de cultură</t>
@@ -1089,7 +1216,11 @@
       <c r="E33" t="n">
         <v>3</v>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G33" s="3" t="n">
         <v>98.90000000000001</v>
       </c>
@@ -1108,7 +1239,11 @@
       <c r="E34" t="n">
         <v>3</v>
       </c>
-      <c r="F34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G34" s="3" t="n">
         <v>188.31</v>
       </c>
@@ -1127,7 +1262,11 @@
       <c r="E35" t="n">
         <v>3</v>
       </c>
-      <c r="F35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G35" s="3" t="n">
         <v>148.31</v>
       </c>
@@ -1146,7 +1285,11 @@
       <c r="E36" t="n">
         <v>3</v>
       </c>
-      <c r="F36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G36" s="3" t="n">
         <v>40</v>
       </c>
@@ -1165,7 +1308,11 @@
       <c r="E37" t="n">
         <v>3</v>
       </c>
-      <c r="F37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G37" s="3" t="n">
         <v>14263</v>
       </c>
@@ -1184,7 +1331,11 @@
       <c r="E38" t="n">
         <v>3</v>
       </c>
-      <c r="F38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G38" s="3" t="n">
         <v>6386</v>
       </c>
@@ -1203,7 +1354,11 @@
       <c r="E39" t="n">
         <v>3</v>
       </c>
-      <c r="F39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G39" s="3" t="n">
         <v>1690</v>
       </c>
@@ -1222,7 +1377,11 @@
       <c r="E40" t="n">
         <v>3</v>
       </c>
-      <c r="F40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G40" s="3" t="n">
         <v>6187</v>
       </c>
@@ -1241,7 +1400,11 @@
       <c r="E41" t="n">
         <v>3</v>
       </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G41" s="3" t="n">
         <v>4000</v>
       </c>
@@ -1260,7 +1423,11 @@
       <c r="E42" t="n">
         <v>3</v>
       </c>
-      <c r="F42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G42" s="3" t="n">
         <v>1520</v>
       </c>
@@ -1279,7 +1446,11 @@
       <c r="E43" t="n">
         <v>3</v>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G43" s="3" t="n">
         <v>800</v>
       </c>
@@ -1298,7 +1469,11 @@
       <c r="E44" t="n">
         <v>3</v>
       </c>
-      <c r="F44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G44" s="3" t="n">
         <v>5133.84</v>
       </c>
@@ -1317,7 +1492,11 @@
       <c r="E45" t="n">
         <v>3</v>
       </c>
-      <c r="F45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G45" s="3" t="n">
         <v>50430</v>
       </c>
@@ -1336,7 +1515,11 @@
       <c r="E46" t="n">
         <v>3</v>
       </c>
-      <c r="F46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G46" s="3" t="n">
         <v>21914</v>
       </c>
@@ -1355,7 +1538,11 @@
       <c r="E47" t="n">
         <v>3</v>
       </c>
-      <c r="F47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G47" s="3" t="n">
         <v>556</v>
       </c>
@@ -1365,7 +1552,7 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="30" customHeight="1">
       <c r="C48" s="2" t="inlineStr">
         <is>
           <t>- Aparat propriu Direcția de Asistență Socială, Centrul de zi, centrul de noapte</t>
@@ -1374,7 +1561,11 @@
       <c r="E48" t="n">
         <v>3</v>
       </c>
-      <c r="F48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G48" s="3" t="n">
         <v>5358</v>
       </c>
@@ -1393,7 +1584,11 @@
       <c r="E49" t="n">
         <v>3</v>
       </c>
-      <c r="F49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G49" s="3" t="n">
         <v>16000</v>
       </c>
@@ -1412,7 +1607,11 @@
       <c r="E50" t="n">
         <v>3</v>
       </c>
-      <c r="F50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G50" s="3" t="n">
         <v>2839</v>
       </c>
@@ -1431,7 +1630,11 @@
       <c r="E51" t="n">
         <v>3</v>
       </c>
-      <c r="F51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G51" s="3" t="n">
         <v>1644</v>
       </c>
@@ -1441,7 +1644,7 @@
         </is>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="30" customHeight="1">
       <c r="C52" s="2" t="inlineStr">
         <is>
           <t>- Aparat propiu Direcția de Asistență Socială, Centrul de zi, centrul de noapte</t>
@@ -1450,7 +1653,11 @@
       <c r="E52" t="n">
         <v>3</v>
       </c>
-      <c r="F52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G52" s="3" t="n">
         <v>1195</v>
       </c>
@@ -1460,7 +1667,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="30" customHeight="1">
       <c r="C53" s="2" t="inlineStr">
         <is>
           <t>- contribuție persoane cu handicap neangajate* Direcția de Asistență Socială</t>
@@ -1469,7 +1676,11 @@
       <c r="E53" t="n">
         <v>3</v>
       </c>
-      <c r="F53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G53" s="3" t="n">
         <v>450</v>
       </c>
@@ -1479,7 +1690,7 @@
         </is>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="30" customHeight="1">
       <c r="C54" s="2" t="inlineStr">
         <is>
           <t>-ajutor incalzire - Legea consumatorului vulnerabil - supliment energie, ajutor încălzire lemne</t>
@@ -1488,7 +1699,11 @@
       <c r="E54" t="n">
         <v>4</v>
       </c>
-      <c r="F54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G54" s="3" t="n">
         <v>552</v>
       </c>
@@ -1507,7 +1722,11 @@
       <c r="E55" t="n">
         <v>4</v>
       </c>
-      <c r="F55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G55" s="3" t="n">
         <v>22946</v>
       </c>
@@ -1526,7 +1745,11 @@
       <c r="E56" t="n">
         <v>4</v>
       </c>
-      <c r="F56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G56" s="3" t="n">
         <v>744</v>
       </c>
@@ -1536,7 +1759,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="30" customHeight="1">
       <c r="C57" s="2" t="inlineStr">
         <is>
           <t>- finanțare programe sociale - tichete cadou pentru cheltuieli sociale</t>
@@ -1545,7 +1768,11 @@
       <c r="E57" t="n">
         <v>4</v>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G57" s="3" t="n">
         <v>900</v>
       </c>
@@ -1564,7 +1791,11 @@
       <c r="E58" t="n">
         <v>4</v>
       </c>
-      <c r="F58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G58" s="3" t="n">
         <v>85</v>
       </c>
@@ -1577,13 +1808,17 @@
     <row r="59">
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>SERVICII ŞI DEZVOLTARE PUBLICÃ SI LOCUINTE, total- din care:</t>
+          <t>SERVICII SI DEZVOLTARE PUBLICÃ SI LOCUINTE, total- din care:</t>
         </is>
       </c>
       <c r="E59" t="n">
         <v>4</v>
       </c>
-      <c r="F59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G59" s="3" t="n">
         <v>14529.16</v>
       </c>
@@ -1602,7 +1837,11 @@
       <c r="E60" t="n">
         <v>4</v>
       </c>
-      <c r="F60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G60" s="3" t="n">
         <v>8200</v>
       </c>
@@ -1612,7 +1851,7 @@
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="30" customHeight="1">
       <c r="C61" s="2" t="inlineStr">
         <is>
           <t>- iluminat public mentenanta, obiecte de inventar, inchiriere iluminat ornamental</t>
@@ -1621,7 +1860,11 @@
       <c r="E61" t="n">
         <v>4</v>
       </c>
-      <c r="F61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G61" s="3" t="n">
         <v>4900</v>
       </c>
@@ -1640,7 +1883,11 @@
       <c r="E62" t="n">
         <v>4</v>
       </c>
-      <c r="F62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G62" s="3" t="n">
         <v>3300</v>
       </c>
@@ -1650,7 +1897,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="30" customHeight="1">
       <c r="C63" s="2" t="inlineStr">
         <is>
           <t>- transferuri Direcția Servicii Publice pentru administrarea Piețelor Oborului și Cimitirelor</t>
@@ -1659,7 +1906,11 @@
       <c r="E63" t="n">
         <v>4</v>
       </c>
-      <c r="F63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G63" s="3" t="n">
         <v>500</v>
       </c>
@@ -1669,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="30" customHeight="1">
       <c r="C64" s="2" t="inlineStr">
         <is>
           <t>- transferuri Direcția Servicii Publice pentru activitatea de intervenții edilitare</t>
@@ -1678,7 +1929,11 @@
       <c r="E64" t="n">
         <v>4</v>
       </c>
-      <c r="F64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G64" s="3" t="n">
         <v>5829.16</v>
       </c>
@@ -1697,7 +1952,11 @@
       <c r="E65" t="n">
         <v>4</v>
       </c>
-      <c r="F65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G65" s="3" t="n">
         <v>41049.12</v>
       </c>
@@ -1716,7 +1975,11 @@
       <c r="E66" t="n">
         <v>4</v>
       </c>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G66" s="3" t="n">
         <v>39849.12</v>
       </c>
@@ -1735,7 +1998,11 @@
       <c r="E67" t="n">
         <v>4</v>
       </c>
-      <c r="F67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G67" s="3" t="n">
         <v>14183.32</v>
       </c>
@@ -1745,7 +2012,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="30" customHeight="1">
       <c r="C68" s="2" t="inlineStr">
         <is>
           <t>- întreținerea albiilor râurilor, Dezinsecție Deratizare Dezinfecție, depozite necontrolate</t>
@@ -1754,7 +2021,11 @@
       <c r="E68" t="n">
         <v>4</v>
       </c>
-      <c r="F68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G68" s="3" t="n">
         <v>300</v>
       </c>
@@ -1773,7 +2044,11 @@
       <c r="E69" t="n">
         <v>4</v>
       </c>
-      <c r="F69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G69" s="3" t="n">
         <v>316.8</v>
       </c>
@@ -1786,13 +2061,17 @@
     <row r="70">
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>- colectare deșeuri (transport gunoi menajer)</t>
+          <t>- colectare deşeuri (transport gunoi menajer)</t>
         </is>
       </c>
       <c r="E70" t="n">
         <v>4</v>
       </c>
-      <c r="F70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G70" s="3" t="n">
         <v>20594</v>
       </c>
@@ -1805,13 +2084,17 @@
     <row r="71">
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>- canalizare (apa pluvială)</t>
+          <t>- canalizare (apa pluvialã)</t>
         </is>
       </c>
       <c r="E71" t="n">
         <v>4</v>
       </c>
-      <c r="F71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G71" s="3" t="n">
         <v>4455</v>
       </c>
@@ -1830,7 +2113,11 @@
       <c r="E72" t="n">
         <v>4</v>
       </c>
-      <c r="F72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G72" s="3" t="n">
         <v>1200</v>
       </c>
@@ -1849,7 +2136,11 @@
       <c r="E73" t="n">
         <v>4</v>
       </c>
-      <c r="F73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G73" s="3" t="n">
         <v>7000</v>
       </c>
@@ -1868,7 +2159,11 @@
       <c r="E74" t="n">
         <v>4</v>
       </c>
-      <c r="F74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G74" s="3" t="n">
         <v>7000</v>
       </c>
@@ -1887,7 +2182,11 @@
       <c r="E75" t="n">
         <v>4</v>
       </c>
-      <c r="F75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G75" s="3" t="n">
         <v>36257.44</v>
       </c>
@@ -1906,7 +2205,11 @@
       <c r="E76" t="n">
         <v>4</v>
       </c>
-      <c r="F76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G76" s="3" t="n">
         <v>25130</v>
       </c>
@@ -1925,7 +2228,11 @@
       <c r="E77" t="n">
         <v>4</v>
       </c>
-      <c r="F77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G77" s="3" t="n">
         <v>24900</v>
       </c>
@@ -1944,7 +2251,11 @@
       <c r="E78" t="n">
         <v>4</v>
       </c>
-      <c r="F78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G78" s="3" t="n">
         <v>230</v>
       </c>
@@ -1963,7 +2274,11 @@
       <c r="E79" t="n">
         <v>4</v>
       </c>
-      <c r="F79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G79" s="3" t="n">
         <v>11827.44</v>
       </c>
@@ -1982,7 +2297,11 @@
       <c r="E80" t="n">
         <v>4</v>
       </c>
-      <c r="F80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G80" s="3" t="n">
         <v>6884.14</v>
       </c>
@@ -2001,7 +2320,11 @@
       <c r="E81" t="n">
         <v>4</v>
       </c>
-      <c r="F81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G81" s="3" t="n">
         <v>4243.3</v>
       </c>
@@ -2020,7 +2343,11 @@
       <c r="E82" t="n">
         <v>4</v>
       </c>
-      <c r="F82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G82" s="3" t="n">
         <v>289516.79</v>
       </c>
@@ -2103,7 +2430,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Fisier</t>
         </is>
@@ -2115,17 +2442,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Schema calitate</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Metrica de calitate</t>
         </is>
@@ -2137,7 +2464,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Recall masurat</t>
         </is>
@@ -2149,7 +2476,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Documente</t>
         </is>
@@ -2159,67 +2486,67 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Linii de date</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Linii strict verificate</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>% linii strict verificate</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Celule numerice</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Celule numerice strict verificate</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>% celule numerice strict verificate</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Pagini asteptate</t>
         </is>
@@ -2229,7 +2556,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Pagini selectate</t>
         </is>
@@ -2239,7 +2566,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Pagini procesate</t>
         </is>
@@ -2249,7 +2576,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>PDF complet</t>
         </is>
@@ -2261,27 +2588,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Linii fara probleme</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>% curat</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Erori</t>
         </is>
@@ -2291,7 +2618,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Avertismente</t>
         </is>
@@ -2301,7 +2628,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Informatii</t>
         </is>
@@ -2311,7 +2638,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Schema publicare</t>
         </is>
@@ -2321,19 +2648,19 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Bundle conversie</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>196ff61ca686343b66bb95ae</t>
+          <t>16df794beae27def1837085d</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>SHA-256 PDF sursa</t>
         </is>
@@ -2345,7 +2672,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>— Anexa (de la pagina 2)</t>
         </is>

</xml_diff>

<commit_message>
feat: complete deterministic PDF extraction P1 (#15)
Co-authored-by: Dan Paraschiv <dan.paraschiv@gmail.com>
</commit_message>
<xml_diff>
--- a/data/2025/07-botosani/35731-botosani/budget_file.xlsx
+++ b/data/2025/07-botosani/35731-botosani/budget_file.xlsx
@@ -60,11 +60,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +438,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -477,7 +480,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL 2026</t>
+          <t>TOTAL 2025</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -500,7 +503,11 @@
       <c r="E2" t="n">
         <v>2</v>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G2" s="3" t="n">
         <v>42303</v>
       </c>
@@ -510,7 +517,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="30" customHeight="1">
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>- cheltuieli de personal aparatul de specialitate al primarului, consilieri locali și aparatul Consiliului Local</t>
@@ -519,7 +526,11 @@
       <c r="E3" t="n">
         <v>2</v>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G3" s="3" t="n">
         <v>28749</v>
       </c>
@@ -529,16 +540,20 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="75" customHeight="1">
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>- bunuri si servicii - cheltuielile curente de întreținere și funcționare a spațiilor unde îşi desfăşoară activitatea personalul Primăriei Municipiului Botoşani (iluminat și încălzire, materiale de întreținere și curățenie, apă-canal, telefoane, furnituri de birou, service programe informatice, mentenanță, costuri pentru medicina muncii).</t>
+          <t>- bunuri si servici - cheltuielile curente de întreținere și funcționare a spațiilor unde îşi desfăşoară activitatea personalul Primăriei Municipiului Botoşani (iluminat și încălzire, materiale de întreținere și curățenie, apã-canal, telefoane, furnituri de birou, service programe informatice, mentenanță, costuri pentru medicina muncii).</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>2</v>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G4" s="3" t="n">
         <v>4225</v>
       </c>
@@ -557,7 +572,11 @@
       <c r="E5" t="n">
         <v>2</v>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="n">
         <v>285</v>
       </c>
@@ -576,7 +595,11 @@
       <c r="E6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="n">
         <v>9044</v>
       </c>
@@ -595,7 +618,11 @@
       <c r="E7" t="n">
         <v>2</v>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G7" s="3" t="n">
         <v>4215.5</v>
       </c>
@@ -605,7 +632,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="30" customHeight="1">
       <c r="C8" s="2" t="inlineStr">
         <is>
           <t>- cheltuieli de personal Serviciul Public Comunitar de Evidență a Persoanelor</t>
@@ -614,7 +641,11 @@
       <c r="E8" t="n">
         <v>2</v>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G8" s="3" t="n">
         <v>2500.5</v>
       </c>
@@ -624,7 +655,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="30" customHeight="1">
       <c r="C9" s="2" t="inlineStr">
         <is>
           <t>- bunuri si servicii Serviciul Public Comunitar de Evidență a Persoanelor</t>
@@ -633,7 +664,11 @@
       <c r="E9" t="n">
         <v>2</v>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G9" s="3" t="n">
         <v>215</v>
       </c>
@@ -643,16 +678,20 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="75" customHeight="1">
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>- cotizații AsociațiaMunicipiilor, Zona Metropolitană, Asociația G.A.L., sprijin viager pentru persoanele care au împlinit vârsta de 85 de ani, sume acordate pentru cuplurile care au împlinit 50 respectiv 60 de ani de căsătorie, executarea silită a creanțelor bugetare, oraganizare evenimente cu ocazia zilei oraşului, zilei de 1 iunie, sărbători de iarnă</t>
+          <t>- cotizații Asociația Municipiilor, Zona Metropolitană, Asociația G.A.L., sprijin viager pentru persoanele care au împlinit vârsta de 85 de ani, sume acordate pentru cuplurile care au împlinit 50 respectiv 60 de ani de căsătorie, executarea silită a creanțelor bugetare, oraganizare evenimente cu ocazia zilei oraşului, zilei de 1 iunie, sărbători de iarnă</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>2</v>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G10" s="3" t="n">
         <v>1500</v>
       </c>
@@ -671,7 +710,11 @@
       <c r="E11" t="n">
         <v>2</v>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G11" s="3" t="n">
         <v>5</v>
       </c>
@@ -690,7 +733,11 @@
       <c r="E12" t="n">
         <v>2</v>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G12" s="3" t="n">
         <v>9725</v>
       </c>
@@ -709,7 +756,11 @@
       <c r="E13" t="n">
         <v>2</v>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G13" s="3" t="n">
         <v>9725</v>
       </c>
@@ -728,7 +779,11 @@
       <c r="E14" t="n">
         <v>2</v>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G14" s="3" t="n">
         <v>11172.25</v>
       </c>
@@ -738,7 +793,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="30" customHeight="1">
       <c r="C15" s="2" t="inlineStr">
         <is>
           <t>- cheltuieli de personal Serviciul Voluntar pentru Situații de Urgență</t>
@@ -747,7 +802,11 @@
       <c r="E15" t="n">
         <v>2</v>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G15" s="3" t="n">
         <v>140</v>
       </c>
@@ -757,7 +816,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="30" customHeight="1">
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>- bunuri si servicii Serviciul Voluntar pentru Situații de Urgență</t>
@@ -766,7 +825,11 @@
       <c r="E16" t="n">
         <v>2</v>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G16" s="3" t="n">
         <v>43</v>
       </c>
@@ -776,7 +839,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="30" customHeight="1">
       <c r="C17" s="2" t="inlineStr">
         <is>
           <t>- transferuri pentru Poliția Locală (în completarea veniturilor proprii ale instituției)</t>
@@ -785,7 +848,11 @@
       <c r="E17" t="n">
         <v>2</v>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G17" s="3" t="n">
         <v>10989.25</v>
       </c>
@@ -798,13 +865,17 @@
     <row r="18">
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>ÎNVÅTÄMÂNT -total, din care:</t>
+          <t>ÎNVÅTÅMÂNT -total, din care:</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>2</v>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G18" s="3" t="n">
         <v>37388.52</v>
       </c>
@@ -814,7 +885,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="30" customHeight="1">
       <c r="C19" s="2" t="inlineStr">
         <is>
           <t>- finantare de bază în baza costului pe elev și transport elevi</t>
@@ -823,7 +894,11 @@
       <c r="E19" t="n">
         <v>2</v>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G19" s="3" t="n">
         <v>20421</v>
       </c>
@@ -842,7 +917,11 @@
       <c r="E20" t="n">
         <v>2</v>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G20" s="3" t="n">
         <v>2266.52</v>
       </c>
@@ -852,7 +931,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="45" customHeight="1">
       <c r="C21" s="2" t="inlineStr">
         <is>
           <t>- tichete grădiniță - finanțarea drepturilor stabilite de Legea nr.248/2015 privind stimularea participării în învățământul preşcolar a copiilor provenind din familii defavorizate</t>
@@ -861,7 +940,11 @@
       <c r="E21" t="n">
         <v>2</v>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G21" s="3" t="n">
         <v>120</v>
       </c>
@@ -871,7 +954,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="30" customHeight="1">
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>- finantare invatamant particular acreditat în baza costului standard pe elev</t>
@@ -880,7 +963,11 @@
       <c r="E22" t="n">
         <v>2</v>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G22" s="3" t="n">
         <v>7848</v>
       </c>
@@ -890,16 +977,20 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="75" customHeight="1">
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>- finanțarea drepturilor copilor cu cerințe educaționale speciale integrați în învățământul de masă, prevăzute la lit.A din Anexa la HG 904/2014 privind stabilirea limitelor minime de cheltuieli aferente drepturilor prevăzute la art.129 alin(1) din Legea 272/2004 privind protecția și promovarea drepturilor copiilor</t>
+          <t>- finanțarea drepturilor copiilor cu cerințe educaționale speciale integrați în învățământul de masă, prevăzute la lit.A din Anexa la HG 904/2014 privind stabilirea limitelor minime de cheltuieli aferente drepturilor prevăzute la art.129 alin(1) din Legea 272/2004 privind protecția și promovarea drepturilor copiilor</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>3</v>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G23" s="3" t="n">
         <v>2649</v>
       </c>
@@ -918,7 +1009,11 @@
       <c r="E24" t="n">
         <v>3</v>
       </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G24" s="3" t="n">
         <v>3357</v>
       </c>
@@ -928,7 +1023,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="30" customHeight="1">
       <c r="C25" s="2" t="inlineStr">
         <is>
           <t>- asociatii si fundatii (Asociația Il Girotondo cu care Consiliul Local este partener)</t>
@@ -937,7 +1032,11 @@
       <c r="E25" t="n">
         <v>3</v>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G25" s="3" t="n">
         <v>727</v>
       </c>
@@ -956,7 +1055,11 @@
       <c r="E26" t="n">
         <v>3</v>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G26" s="3" t="n">
         <v>9104.4</v>
       </c>
@@ -966,7 +1069,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="60" customHeight="1">
       <c r="C27" s="2" t="inlineStr">
         <is>
           <t>- cheltuieli de personal finanțarea personalului cabinetelor medicale şcolare și cabinete stomatologice care funcționează în instituțiile de învățământ și a asistenței medicale comunitare</t>
@@ -975,7 +1078,11 @@
       <c r="E27" t="n">
         <v>3</v>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G27" s="3" t="n">
         <v>8736.5</v>
       </c>
@@ -985,16 +1092,20 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="30" customHeight="1">
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>- bunuri si servicii cabinete medicale școlare și cabinete stomatologice care funcționează în instituțiile de învățământ</t>
+          <t>- bunuri si servicii cabinete medicale şcolare și cabinete stomatologice care funcționează în instituțiile de învățământ</t>
         </is>
       </c>
       <c r="E28" t="n">
         <v>3</v>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G28" s="3" t="n">
         <v>280.4</v>
       </c>
@@ -1004,7 +1115,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="30" customHeight="1">
       <c r="C29" s="2" t="inlineStr">
         <is>
           <t>- contribuție persoane cu handicap neangajate* cabinete şcolare</t>
@@ -1013,7 +1124,11 @@
       <c r="E29" t="n">
         <v>3</v>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G29" s="3" t="n">
         <v>87.5</v>
       </c>
@@ -1032,7 +1147,11 @@
       <c r="E30" t="n">
         <v>3</v>
       </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G30" s="3" t="n">
         <v>26337.4</v>
       </c>
@@ -1051,7 +1170,11 @@
       <c r="E31" t="n">
         <v>3</v>
       </c>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G31" s="3" t="n">
         <v>432.25</v>
       </c>
@@ -1070,7 +1193,11 @@
       <c r="E32" t="n">
         <v>3</v>
       </c>
-      <c r="F32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G32" s="3" t="n">
         <v>333.35</v>
       </c>
@@ -1080,7 +1207,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="30" customHeight="1">
       <c r="C33" s="2" t="inlineStr">
         <is>
           <t>- Premiul național de poezie "M. Eminescu”, comisii evaluare management instituții de cultură</t>
@@ -1089,7 +1216,11 @@
       <c r="E33" t="n">
         <v>3</v>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G33" s="3" t="n">
         <v>98.90000000000001</v>
       </c>
@@ -1108,7 +1239,11 @@
       <c r="E34" t="n">
         <v>3</v>
       </c>
-      <c r="F34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G34" s="3" t="n">
         <v>188.31</v>
       </c>
@@ -1127,7 +1262,11 @@
       <c r="E35" t="n">
         <v>3</v>
       </c>
-      <c r="F35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G35" s="3" t="n">
         <v>148.31</v>
       </c>
@@ -1146,7 +1285,11 @@
       <c r="E36" t="n">
         <v>3</v>
       </c>
-      <c r="F36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G36" s="3" t="n">
         <v>40</v>
       </c>
@@ -1165,7 +1308,11 @@
       <c r="E37" t="n">
         <v>3</v>
       </c>
-      <c r="F37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G37" s="3" t="n">
         <v>14263</v>
       </c>
@@ -1184,7 +1331,11 @@
       <c r="E38" t="n">
         <v>3</v>
       </c>
-      <c r="F38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G38" s="3" t="n">
         <v>6386</v>
       </c>
@@ -1203,7 +1354,11 @@
       <c r="E39" t="n">
         <v>3</v>
       </c>
-      <c r="F39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G39" s="3" t="n">
         <v>1690</v>
       </c>
@@ -1222,7 +1377,11 @@
       <c r="E40" t="n">
         <v>3</v>
       </c>
-      <c r="F40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G40" s="3" t="n">
         <v>6187</v>
       </c>
@@ -1241,7 +1400,11 @@
       <c r="E41" t="n">
         <v>3</v>
       </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G41" s="3" t="n">
         <v>4000</v>
       </c>
@@ -1260,7 +1423,11 @@
       <c r="E42" t="n">
         <v>3</v>
       </c>
-      <c r="F42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G42" s="3" t="n">
         <v>1520</v>
       </c>
@@ -1279,7 +1446,11 @@
       <c r="E43" t="n">
         <v>3</v>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G43" s="3" t="n">
         <v>800</v>
       </c>
@@ -1298,7 +1469,11 @@
       <c r="E44" t="n">
         <v>3</v>
       </c>
-      <c r="F44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G44" s="3" t="n">
         <v>5133.84</v>
       </c>
@@ -1317,7 +1492,11 @@
       <c r="E45" t="n">
         <v>3</v>
       </c>
-      <c r="F45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G45" s="3" t="n">
         <v>50430</v>
       </c>
@@ -1336,7 +1515,11 @@
       <c r="E46" t="n">
         <v>3</v>
       </c>
-      <c r="F46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G46" s="3" t="n">
         <v>21914</v>
       </c>
@@ -1355,7 +1538,11 @@
       <c r="E47" t="n">
         <v>3</v>
       </c>
-      <c r="F47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G47" s="3" t="n">
         <v>556</v>
       </c>
@@ -1365,7 +1552,7 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="30" customHeight="1">
       <c r="C48" s="2" t="inlineStr">
         <is>
           <t>- Aparat propriu Direcția de Asistență Socială, Centrul de zi, centrul de noapte</t>
@@ -1374,7 +1561,11 @@
       <c r="E48" t="n">
         <v>3</v>
       </c>
-      <c r="F48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G48" s="3" t="n">
         <v>5358</v>
       </c>
@@ -1393,7 +1584,11 @@
       <c r="E49" t="n">
         <v>3</v>
       </c>
-      <c r="F49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G49" s="3" t="n">
         <v>16000</v>
       </c>
@@ -1412,7 +1607,11 @@
       <c r="E50" t="n">
         <v>3</v>
       </c>
-      <c r="F50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G50" s="3" t="n">
         <v>2839</v>
       </c>
@@ -1431,7 +1630,11 @@
       <c r="E51" t="n">
         <v>3</v>
       </c>
-      <c r="F51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G51" s="3" t="n">
         <v>1644</v>
       </c>
@@ -1441,7 +1644,7 @@
         </is>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="30" customHeight="1">
       <c r="C52" s="2" t="inlineStr">
         <is>
           <t>- Aparat propiu Direcția de Asistență Socială, Centrul de zi, centrul de noapte</t>
@@ -1450,7 +1653,11 @@
       <c r="E52" t="n">
         <v>3</v>
       </c>
-      <c r="F52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G52" s="3" t="n">
         <v>1195</v>
       </c>
@@ -1460,7 +1667,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="30" customHeight="1">
       <c r="C53" s="2" t="inlineStr">
         <is>
           <t>- contribuție persoane cu handicap neangajate* Direcția de Asistență Socială</t>
@@ -1469,7 +1676,11 @@
       <c r="E53" t="n">
         <v>3</v>
       </c>
-      <c r="F53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G53" s="3" t="n">
         <v>450</v>
       </c>
@@ -1479,7 +1690,7 @@
         </is>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="30" customHeight="1">
       <c r="C54" s="2" t="inlineStr">
         <is>
           <t>-ajutor incalzire - Legea consumatorului vulnerabil - supliment energie, ajutor încălzire lemne</t>
@@ -1488,7 +1699,11 @@
       <c r="E54" t="n">
         <v>4</v>
       </c>
-      <c r="F54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G54" s="3" t="n">
         <v>552</v>
       </c>
@@ -1507,7 +1722,11 @@
       <c r="E55" t="n">
         <v>4</v>
       </c>
-      <c r="F55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G55" s="3" t="n">
         <v>22946</v>
       </c>
@@ -1526,7 +1745,11 @@
       <c r="E56" t="n">
         <v>4</v>
       </c>
-      <c r="F56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G56" s="3" t="n">
         <v>744</v>
       </c>
@@ -1536,7 +1759,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="30" customHeight="1">
       <c r="C57" s="2" t="inlineStr">
         <is>
           <t>- finanțare programe sociale - tichete cadou pentru cheltuieli sociale</t>
@@ -1545,7 +1768,11 @@
       <c r="E57" t="n">
         <v>4</v>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G57" s="3" t="n">
         <v>900</v>
       </c>
@@ -1564,7 +1791,11 @@
       <c r="E58" t="n">
         <v>4</v>
       </c>
-      <c r="F58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G58" s="3" t="n">
         <v>85</v>
       </c>
@@ -1577,13 +1808,17 @@
     <row r="59">
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>SERVICII ŞI DEZVOLTARE PUBLICÃ SI LOCUINTE, total- din care:</t>
+          <t>SERVICII SI DEZVOLTARE PUBLICÃ SI LOCUINTE, total- din care:</t>
         </is>
       </c>
       <c r="E59" t="n">
         <v>4</v>
       </c>
-      <c r="F59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G59" s="3" t="n">
         <v>14529.16</v>
       </c>
@@ -1602,7 +1837,11 @@
       <c r="E60" t="n">
         <v>4</v>
       </c>
-      <c r="F60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G60" s="3" t="n">
         <v>8200</v>
       </c>
@@ -1612,7 +1851,7 @@
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="30" customHeight="1">
       <c r="C61" s="2" t="inlineStr">
         <is>
           <t>- iluminat public mentenanta, obiecte de inventar, inchiriere iluminat ornamental</t>
@@ -1621,7 +1860,11 @@
       <c r="E61" t="n">
         <v>4</v>
       </c>
-      <c r="F61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G61" s="3" t="n">
         <v>4900</v>
       </c>
@@ -1640,7 +1883,11 @@
       <c r="E62" t="n">
         <v>4</v>
       </c>
-      <c r="F62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G62" s="3" t="n">
         <v>3300</v>
       </c>
@@ -1650,7 +1897,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="30" customHeight="1">
       <c r="C63" s="2" t="inlineStr">
         <is>
           <t>- transferuri Direcția Servicii Publice pentru administrarea Piețelor Oborului și Cimitirelor</t>
@@ -1659,7 +1906,11 @@
       <c r="E63" t="n">
         <v>4</v>
       </c>
-      <c r="F63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G63" s="3" t="n">
         <v>500</v>
       </c>
@@ -1669,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="30" customHeight="1">
       <c r="C64" s="2" t="inlineStr">
         <is>
           <t>- transferuri Direcția Servicii Publice pentru activitatea de intervenții edilitare</t>
@@ -1678,7 +1929,11 @@
       <c r="E64" t="n">
         <v>4</v>
       </c>
-      <c r="F64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G64" s="3" t="n">
         <v>5829.16</v>
       </c>
@@ -1697,7 +1952,11 @@
       <c r="E65" t="n">
         <v>4</v>
       </c>
-      <c r="F65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G65" s="3" t="n">
         <v>41049.12</v>
       </c>
@@ -1716,7 +1975,11 @@
       <c r="E66" t="n">
         <v>4</v>
       </c>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G66" s="3" t="n">
         <v>39849.12</v>
       </c>
@@ -1735,7 +1998,11 @@
       <c r="E67" t="n">
         <v>4</v>
       </c>
-      <c r="F67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G67" s="3" t="n">
         <v>14183.32</v>
       </c>
@@ -1745,7 +2012,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="30" customHeight="1">
       <c r="C68" s="2" t="inlineStr">
         <is>
           <t>- întreținerea albiilor râurilor, Dezinsecție Deratizare Dezinfecție, depozite necontrolate</t>
@@ -1754,7 +2021,11 @@
       <c r="E68" t="n">
         <v>4</v>
       </c>
-      <c r="F68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G68" s="3" t="n">
         <v>300</v>
       </c>
@@ -1773,7 +2044,11 @@
       <c r="E69" t="n">
         <v>4</v>
       </c>
-      <c r="F69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G69" s="3" t="n">
         <v>316.8</v>
       </c>
@@ -1786,13 +2061,17 @@
     <row r="70">
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>- colectare deșeuri (transport gunoi menajer)</t>
+          <t>- colectare deşeuri (transport gunoi menajer)</t>
         </is>
       </c>
       <c r="E70" t="n">
         <v>4</v>
       </c>
-      <c r="F70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G70" s="3" t="n">
         <v>20594</v>
       </c>
@@ -1805,13 +2084,17 @@
     <row r="71">
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>- canalizare (apa pluvială)</t>
+          <t>- canalizare (apa pluvialã)</t>
         </is>
       </c>
       <c r="E71" t="n">
         <v>4</v>
       </c>
-      <c r="F71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G71" s="3" t="n">
         <v>4455</v>
       </c>
@@ -1830,7 +2113,11 @@
       <c r="E72" t="n">
         <v>4</v>
       </c>
-      <c r="F72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G72" s="3" t="n">
         <v>1200</v>
       </c>
@@ -1849,7 +2136,11 @@
       <c r="E73" t="n">
         <v>4</v>
       </c>
-      <c r="F73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G73" s="3" t="n">
         <v>7000</v>
       </c>
@@ -1868,7 +2159,11 @@
       <c r="E74" t="n">
         <v>4</v>
       </c>
-      <c r="F74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G74" s="3" t="n">
         <v>7000</v>
       </c>
@@ -1887,7 +2182,11 @@
       <c r="E75" t="n">
         <v>4</v>
       </c>
-      <c r="F75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G75" s="3" t="n">
         <v>36257.44</v>
       </c>
@@ -1906,7 +2205,11 @@
       <c r="E76" t="n">
         <v>4</v>
       </c>
-      <c r="F76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G76" s="3" t="n">
         <v>25130</v>
       </c>
@@ -1925,7 +2228,11 @@
       <c r="E77" t="n">
         <v>4</v>
       </c>
-      <c r="F77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G77" s="3" t="n">
         <v>24900</v>
       </c>
@@ -1944,7 +2251,11 @@
       <c r="E78" t="n">
         <v>4</v>
       </c>
-      <c r="F78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G78" s="3" t="n">
         <v>230</v>
       </c>
@@ -1963,7 +2274,11 @@
       <c r="E79" t="n">
         <v>4</v>
       </c>
-      <c r="F79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G79" s="3" t="n">
         <v>11827.44</v>
       </c>
@@ -1982,7 +2297,11 @@
       <c r="E80" t="n">
         <v>4</v>
       </c>
-      <c r="F80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G80" s="3" t="n">
         <v>6884.14</v>
       </c>
@@ -2001,7 +2320,11 @@
       <c r="E81" t="n">
         <v>4</v>
       </c>
-      <c r="F81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G81" s="3" t="n">
         <v>4243.3</v>
       </c>
@@ -2020,7 +2343,11 @@
       <c r="E82" t="n">
         <v>4</v>
       </c>
-      <c r="F82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>annex</t>
+        </is>
+      </c>
       <c r="G82" s="3" t="n">
         <v>289516.79</v>
       </c>
@@ -2103,7 +2430,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Fisier</t>
         </is>
@@ -2115,17 +2442,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Schema calitate</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Metrica de calitate</t>
         </is>
@@ -2137,7 +2464,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Recall masurat</t>
         </is>
@@ -2149,7 +2476,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Documente</t>
         </is>
@@ -2159,67 +2486,67 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Linii de date</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Linii strict verificate</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>% linii strict verificate</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Celule numerice</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Celule numerice strict verificate</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>% celule numerice strict verificate</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Pagini asteptate</t>
         </is>
@@ -2229,7 +2556,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Pagini selectate</t>
         </is>
@@ -2239,7 +2566,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Pagini procesate</t>
         </is>
@@ -2249,7 +2576,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>PDF complet</t>
         </is>
@@ -2261,27 +2588,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Linii fara probleme</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>% curat</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Erori</t>
         </is>
@@ -2291,7 +2618,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Avertismente</t>
         </is>
@@ -2301,7 +2628,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Informatii</t>
         </is>
@@ -2311,7 +2638,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Schema publicare</t>
         </is>
@@ -2321,19 +2648,19 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Bundle conversie</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>196ff61ca686343b66bb95ae</t>
+          <t>16df794beae27def1837085d</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>SHA-256 PDF sursa</t>
         </is>
@@ -2345,7 +2672,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>— Anexa (de la pagina 2)</t>
         </is>

</xml_diff>